<commit_message>
Record the puja checks on the phone.
The 21-count stays off the practice log, ticks survive a restart, and the offering page hides Search when the phone is offline.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/M3-puja.xlsx
+++ b/tests/M3-puja.xlsx
@@ -652,6 +652,11 @@
       </c>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Pre, During and Post jump to those parts of the puja.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="57.95" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -697,6 +702,11 @@
       </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Durva shows No Durva grass? Akshata (rice with turmeric) is fine. The other items show the same kind of line.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="57.95" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -743,6 +753,11 @@
       </c>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. A durva tick was still there after the app was force-stopped. Clear ticks removed it.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="57.95" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -833,6 +848,11 @@
       </c>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. The patra step reached 21 of 21. Leaving the puja and opening it again showed 0 of 21. Practice totals stayed 112, 7 and 5.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="57.95" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -878,6 +898,11 @@
       </c>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Guided mode shows one step at a time, with Previous and Next, and the screen stays on. Seen at step 24 of 32.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="57.95" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -923,6 +948,11 @@
       </c>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Opening guided mode again asked Continue from step 24.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="57.95" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -968,6 +998,11 @@
       </c>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Telangana leads with Undrallu. Maharashtra leads with Modak. All five forms are on the page. The city was set back to Hyderabad.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="57.95" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1012,6 +1047,11 @@
       </c>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. The page has Why this offering, Offered on (Sankashti, Vinayaka Chavithi, and the puja), and the elder line.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="57.95" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1059,7 +1099,7 @@
       <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not reached. The offering page was not opened while airplane mode was on.</t>
+          <t xml:space="preserve">PASS. Search is on the page while the phone is online. With airplane mode and no network, the page still opens and Search is hidden.</t>
         </is>
       </c>
     </row>
@@ -1107,6 +1147,11 @@
       </c>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. The 21 taps were not written. The japam totals were the same afterwards.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="57.95" customHeight="1">
       <c r="A15" s="3" t="n">

</xml_diff>

<commit_message>
Guided puja audio + hands-free
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/M3-puja.xlsx
+++ b/tests/M3-puja.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -1546,6 +1546,642 @@
         </is>
       </c>
     </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two-part step</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two-part step</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A guided step plays the instruction, then the mantra</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open Vinayaka Chavithi guided mode.
+2. On a step that has both recordings, tap Play.</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The instruction plays in the app language, then the mantra plays in Sanskrit. Nothing starts until Play is tapped.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word lighting</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word lighting</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The mantra word that is being read is lit</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Play a mantra step.
+2. Watch the mantra line.</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each word is lit as it is read, in the script on screen.</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script switch mid-step</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script switch mid-step</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The script can change while the mantra is playing</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Play a mantra step.
+2. While it plays, switch Telugu script, संस्कृतम्, and IAST.</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The line changes script and the lit word stays in place. The audio does not restart.</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">List pause and the count</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">List pause and the count</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The 21 names pause so each offering can be made</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Play the patri step once its list recording is in the pack.
+2. Listen through the names.</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One name is lit at a time. The count reads like 7 of 21. Playback pauses about 3 seconds after each name.</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hands-free countdown</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hands-free countdown</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hands-free moves on, and can be stopped</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. On the guided start screen, leave Hands-free on.
+2. Play a step and let it finish.
+3. While the ring is on Next, try Pause, Back, and a tap on the ring.</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Next shows a 4-second ring, then the next step. Pause freezes it and Play continues it. Back leaves the step and stops the ring. A tap on the ring stops it and stays on the step.</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Katha hands-free round trip</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Katha hands-free round trip</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hands-free plays the Chavithi katha and returns</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. With Hands-free on, play the katha step once both story narrations are in the pack.</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The moon story plays, then the Syamantaka story, then the puja returns and continues.</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Step with no audio waits</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Step with no audio waits</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A step without a recording does not move by itself</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open guided mode before any puja recording is attached.
+2. Leave Hands-free on and look at Next.</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The step keeps Previous and Next, as it does today. Hands-free does not move on until the person taps Next.</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not re-walked. The step keeps Previous and Next, and hands-free waits for Next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lock screen</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lock screen</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Playback continues on the lock screen</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Play a guided step.
+2. Lock the phone.</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The notification reads Step N of 32 · the step title, with Play/Pause and Next. Audio keeps playing.</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Language switch</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Language switch</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Changing language restarts only the instruction</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Play a step's instruction and switch the app language.
+2. Switch language again while the mantra is playing.</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The instruction starts again in the new language. The mantra, once started, keeps playing.</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Telugu, Hindi, and English</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Telugu, Hindi, and English</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The instruction follows the app language</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Play one step in Telugu, Hindi, and English.</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each language plays its own instruction. The mantra stays in Sanskrit.</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200% font</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200% font</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The guided controls still fit</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Set the font scale to 200%.
+2. Open guided mode.</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hands-free, Back, Play, Next, the speed chips, and Repeat step stay tappable. Nothing is clipped to one letter a line.</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TalkBack</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TalkBack</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Play is named for the step</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Turn TalkBack on.
+2. Focus the play control on step 5.</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TalkBack reads Play step 5.</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Airplane mode</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Airplane mode</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guided audio does not need the network</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Turn airplane mode on.
+2. Play a step whose recording is already on the phone.</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The step plays. A step with no recording still waits for Next.</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>